<commit_message>
Obtained a weird spike downward when predicting Tm and Hfus. Test RSME: 0.3108; Train RSME 0.0809
</commit_message>
<xml_diff>
--- a/data/input/MTGPR_Tm_Hfus_Hf/test.xlsx
+++ b/data/input/MTGPR_Tm_Hfus_Hf/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\MTGPR_Tm_Hfus_Hf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28017128-5FDA-4C58-ABC8-F71998D17543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{403DA284-6E7A-4A73-93B1-980C5EFDE836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -434,14 +434,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>3</v>
       </c>
@@ -455,7 +455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -463,24 +463,13 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>397.15</v>
+        <v>402.15</v>
       </c>
       <c r="G2">
-        <f t="shared" ref="G2" si="0">N2/1000</f>
-        <v>15.8</v>
-      </c>
-      <c r="J2">
-        <f t="shared" ref="J2" si="1">O2/1000</f>
-        <v>-395</v>
-      </c>
-      <c r="N2">
-        <v>15800</v>
-      </c>
-      <c r="O2">
-        <v>-395000</v>
+        <v>16.8</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -488,13 +477,10 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <v>381.15</v>
+        <v>384.15</v>
       </c>
       <c r="G3">
-        <v>14.6</v>
-      </c>
-      <c r="J3">
-        <v>-133.4</v>
+        <v>2.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>